<commit_message>
Remove Sales Comparables; scope database to lease & income/expense
Drops the Sales Comparables tab and comp references per scope (lease and
income/expense extraction/storage only). Updates README and the
property-doc-extract skill to skip comps/market-support data going forward.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Fo7yVFxCiBUJva3N3paic
</commit_message>
<xml_diff>
--- a/Master_Property_Database.xlsx
+++ b/Master_Property_Database.xlsx
@@ -13,8 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments &amp; Valuation" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales Comparables" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -661,6 +660,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Tax appeal — income approach + sale comps</t>
+          <t>Tax appeal — income approach</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Appeal of Real Property Valuation — income + market sales</t>
+          <t>Appeal of Real Property Valuation — income approach</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -970,6 +970,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -1053,6 +1054,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2098,6 +2100,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3173,6 +3176,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -3381,6 +3385,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
@@ -3395,6 +3400,7 @@
       <c r="G12" s="20" t="n"/>
       <c r="H12" s="21" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
@@ -3591,6 +3597,7 @@
         <v>2460577</v>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -3648,6 +3655,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3762,12 +3770,17 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Net = Total Income − Total Expense as printed. Bases differ: 5970 Marion &amp; Broadview totals include financing/depreciation, so they are cash-flow / tax figures, not NOI. TempTee reported operating expenses only. See 'Assessments &amp; Valuation' tab for stabilized NOI proformas.</t>
         </is>
       </c>
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3809,6 +3822,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5206,276 +5220,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SALES COMPARABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Warehouse sale comps supporting the R0169133 (17608 E. 24th Dr) appraisal — CoStar / Ryan LLC</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Address</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>City, ST ZIP</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Year Built</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Building SF</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Sale Date</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Sale Price</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Price PSF</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>8495 Roslyn St</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Commerce City, CO 80022</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>1987</v>
-      </c>
-      <c r="F5" s="29" t="n">
-        <v>15100</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>3/25/2024</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>165.56</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>11900 E 33rd Ave</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Aurora, CO 80010</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>1996</v>
-      </c>
-      <c r="F6" s="29" t="n">
-        <v>39655</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>1/23/2024</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>6700000</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>168.96</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>6270 E 50th Ave</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Commerce City, CO 80022</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>1996</v>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>35441</v>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>11/6/2023</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>3775000</v>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>106.52</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>7001 E 57th Pl</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Commerce City, CO 80022</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>1982</v>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>22000</v>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>9/20/2022</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>3685000</v>
-      </c>
-      <c r="I8" s="16" t="n">
-        <v>167.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr"/>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr"/>
-      <c r="D9" s="13" t="inlineStr"/>
-      <c r="E9" s="13" t="inlineStr"/>
-      <c r="F9" s="30">
-        <f>AVERAGE(F5:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="13" t="inlineStr"/>
-      <c r="H9" s="14">
-        <f>AVERAGE(H5:H8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="31">
-        <f>AVERAGE(I5:I8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Source: CoStar (©2025), included in the R0169133 package. Other appeal files also contain comps: R0092302 &amp; 5650 Washington St include CoStar sale/rent comps; R0024442 &amp; R0178308 include CoStar rent/sale sheets — not itemized here (supporting market data).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A11:I11"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5505,6 +5249,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5640,12 +5385,17 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Highlighted row (R0178308 / 7205 Gilpin Way) is the primary appeal subject; the other three parcels are co-listed on the same authorization schedule. Appeal owner of record: Center Land Properties (signed by Ken R. Lombardi, Manager).</t>
         </is>
       </c>
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Add 10350 Washington self-storage comparison + master DB entries
Extracts income/expense and valuation detail for the three Adams County
self-storage tax appeals in the December Hearings / R0040829 - 10350
Washington Street folder: the subject (10350 Washington, R0040829) and
comps 15413 E 18th Ave (R0086010) and 1540 Altura Blvd (R0085571).

- New "Self-Storage Comparison" tab: side-by-side property profile,
  assessed value, income-approach proforma, and actual Dec 2024 YTD
  operating statement (where available) across all three properties.
- Adds the three properties to Source Documents, Property Master,
  Assessments & Valuation, Income-Expense Summary, and Income-Expense
  Detail, with all totals verified against the printed source figures.
- README updated with the new properties and tab.
</commit_message>
<xml_diff>
--- a/Master_Property_Database.xlsx
+++ b/Master_Property_Database.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Documents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property Master" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenants &amp; Leases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments &amp; Valuation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Source Documents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Property Master" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tenants &amp; Leases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Assessments &amp; Valuation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Income-Expense Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Income-Expense Detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Related Parcels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Self-Storage Comparison" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);-"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +75,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +117,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -269,6 +286,73 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -635,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -656,11 +740,10 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared for Carter Equities  |  Updated 2026-07-30  |  8 subject properties, all Adams County, Colorado</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Prepared for Carter Equities  |  Updated 2026-08-19  |  11 subject properties, all Adams County, Colorado</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -970,23 +1053,142 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Appeal docs R0040829.pdf</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Tax appeal - income approach + auth letter (self storage)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington Street (R0040829)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Assess. Yr 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Ryan LLC (D. Fassig) / Dahn Corp (PTA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>R0040829 self storage.pdf</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Duplicate of Appeal docs R0040829.pdf (identical content)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington Street (R0040829)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Assess. Yr 2026</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Ryan LLC (D. Fassig) / Dahn Corp (PTA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>R0086010 - 15413 E 18th Avenue.pdf</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Tax appeal - income approach + actual income statement + abatement petition</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave, Aurora (R0086010)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Assess. Yr 2026 (petition tax yr 2025)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Ryan LLC (D. Fassig) / CubeSmart (store 6730)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>R0085571 - 1540 Altura Blvd.pdf</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Tax appeal - income approach + actual income statement</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd, Aurora (R0085571)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Assess. Yr 2025/2026 (as printed)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Ryan LLC (D. Fassig) / CubeSmart (store 6731)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Notes: Figures transcribed from the source documents. Total / net / average cells are live formulas (SUM/AVERAGE) verified against the printed totals; they populate on open in Excel/Sheets.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>'in house' on the TempTee survey = owner self-performs the service (no $ reported), entered as $0. 5650 Washington St concluded value, rent-roll grid, and income proforma are embedded as EMF vector images in the DOCX and were not text-extractable; narrative figures are captured where stated.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>5970 Marion cash-basis 'expense' includes mortgage P&amp;I and property taxes (cash flow, not NOI). R0169133 cover value ($3,408,546) differs from its schedule total ($3,114,815); both reproduced as printed.</t>
         </is>
@@ -995,10 +1197,10 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1010,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1054,7 +1256,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2049,6 +2250,331 @@
       <c r="Y12" s="6" t="inlineStr">
         <is>
           <t>R0092302.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>R0040829</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>R0040829</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>0171914201013</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Thornton (TH) - Dahn - 21548</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington Street</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Adams</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>DSI Special Situations Fund B</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>DSI Special Situations Fund B</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Specialty - Self Storage</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>Single (proforma; blanket self-storage lease)</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>127395</v>
+      </c>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="n">
+        <v>48250</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>1985</v>
+      </c>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>84% actual / 85% stabilized (Jun 2024)</t>
+        </is>
+      </c>
+      <c r="U13" s="9" t="n">
+        <v>5428808</v>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W13" s="9" t="n">
+        <v>4510000</v>
+      </c>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>Dahn Corporation (PTA)</t>
+        </is>
+      </c>
+      <c r="Y13" s="6" t="inlineStr">
+        <is>
+          <t>Appeal docs R0040829.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>R0086010</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>R0086010</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>0182132318001</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Aurora - 18th Avenue - CS - 6730</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>80011</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Adams</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC / PTA USI No 730</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC / PTA USI No 730</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Specialty - Self Storage</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>Single (proforma; blanket self-storage lease)</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="O14" s="8" t="n">
+        <v>203817</v>
+      </c>
+      <c r="P14" s="8" t="n"/>
+      <c r="Q14" s="8" t="n">
+        <v>57742</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>1984</v>
+      </c>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>87% actual / 88% stabilized (Jun 2024)</t>
+        </is>
+      </c>
+      <c r="U14" s="9" t="n">
+        <v>8187500</v>
+      </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W14" s="9" t="n">
+        <v>6610000</v>
+      </c>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
+          <t>CubeSmart (store 6730)</t>
+        </is>
+      </c>
+      <c r="Y14" s="6" t="inlineStr">
+        <is>
+          <t>R0086010 - 15413 E 18th Avenue.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>R0085571</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>R0085571</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>0182131405022</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Aurora Altura Boulevard CS 6731</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>80011</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Adams</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC / PTA USI No 731</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Specialty - Self Storage</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>Single (proforma; blanket self-storage lease)</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>89298</v>
+      </c>
+      <c r="P15" s="8" t="n"/>
+      <c r="Q15" s="8" t="n">
+        <v>27139</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>1978</v>
+      </c>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>3.29:1</t>
+        </is>
+      </c>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>100% assumed in proforma (0% vacancy loss)</t>
+        </is>
+      </c>
+      <c r="U15" s="9" t="n">
+        <v>3309468</v>
+      </c>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="W15" s="9" t="n">
+        <v>2546900</v>
+      </c>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
+          <t>CubeSmart (store 6731)</t>
+        </is>
+      </c>
+      <c r="Y15" s="6" t="inlineStr">
+        <is>
+          <t>R0085571 - 1540 Altura Blvd.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2626,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3149,7 +3674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3176,7 +3701,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -3385,241 +3909,414 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>5428808</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>112.51</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>4510000</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>R0040829</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>8187500</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>141.79</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>6610000</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>114.47</v>
+      </c>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>R0086010</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>3309468</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>121.95</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>2546900</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>93.84999999999999</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>3571199</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>R0085571</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Historical detail — R0178308: 2025 Land $1,125,150 / Imp $4,025,175 / Total $5,150,325; 2024 Total $4,999,770.  R0169133: 2025 Land $992,519 / Imp $2,122,296 / schedule Total $3,114,815 (cover shows $3,408,546); 2024 Total $2,900,000.  R0024442: 2024 County $2,000,000 → 2025 $3,876,387 (+93.8%).</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="21" t="n"/>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="20" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="20" t="n"/>
+      <c r="F15" s="20" t="n"/>
+      <c r="G15" s="20" t="n"/>
+      <c r="H15" s="21" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>B. Income-Approach Proformas</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="21" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="20" t="n"/>
+      <c r="F17" s="20" t="n"/>
+      <c r="G17" s="20" t="n"/>
+      <c r="H17" s="21" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>PGI</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Vacancy</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>EGI</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Operating Exp</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>NOI</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Cap Rate</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Indicated Value</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>7205 Gilpin Way</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="n">
-        <v>359394</v>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>-17970</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>341424</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>-27314</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>314110</v>
-      </c>
-      <c r="G16" s="19" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="H16" s="14" t="n">
-        <v>4832500</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>17608 E. 24th Dr</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>209100</v>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>-10455</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>198645</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>-15892</v>
-      </c>
-      <c r="F17" s="14" t="n">
-        <v>182753</v>
-      </c>
-      <c r="G17" s="19" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H17" s="14" t="n">
-        <v>3050000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>12260 Pennsylvania St</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>237290</v>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>-16610</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>220680</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>-22068</v>
-      </c>
-      <c r="F18" s="14" t="n">
-        <v>198612</v>
-      </c>
-      <c r="G18" s="19" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="H18" s="14" t="n">
-        <v>2837000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>6770 E. 56th Ave</t>
+          <t>7205 Gilpin Way</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>115824</v>
+        <v>359394</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-5791</v>
+        <v>-17970</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>110033</v>
+        <v>341424</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>-5502</v>
+        <v>-27314</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>104531</v>
+        <v>314110</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="H19" s="14" t="n">
-        <v>1493302</v>
+        <v>4832500</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>17608 E. 24th Dr</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>209100</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>-10455</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>198645</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>-15892</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>182753</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>3050000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>12260 Pennsylvania St</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>237290</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>-16610</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>220680</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>-22068</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>198612</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>2837000</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>6770 E. 56th Ave</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>115824</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>-5791</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>110033</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>-5502</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>104531</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>1493302</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>5970 Marion Drive (mkt)</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B23" s="9" t="n">
         <v>172800</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C23" s="9" t="n">
         <v>-8640</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D23" s="9" t="n">
         <v>164160</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E23" s="9" t="n">
         <v>-4223</v>
       </c>
-      <c r="F20" s="14" t="n">
+      <c r="F23" s="14" t="n">
         <v>159937</v>
       </c>
-      <c r="G20" s="19" t="n">
+      <c r="G23" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="H20" s="14" t="n">
+      <c r="H23" s="14" t="n">
         <v>2460577</v>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Proforma vacancy/EGI figures as reported by each preparer (Ryan, Property Tax Advisors, or owner's analysis). 5970 Marion figures are from the owner's income-approach block in the 2024 P&amp;L workbook (PGI $172,800, 95% occ, NOI $159,938, 6.5% cap → $2,460,577; assigned $2,527,915).</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="n"/>
-      <c r="H22" s="21" t="n"/>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington St (proforma)</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>796125</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>-119419</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>676706</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>-372188</v>
+      </c>
+      <c r="F24" s="32" t="n">
+        <v>304518</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="H24" s="32" t="n">
+        <v>4510000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (proforma)</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>750646</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>-90078</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>660568</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>-231199</v>
+      </c>
+      <c r="F25" s="32" t="n">
+        <v>429370</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H25" s="32" t="n">
+        <v>6610000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (proforma)</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>413870</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>413870</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>-248322</v>
+      </c>
+      <c r="F26" s="32" t="n">
+        <v>165548</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H26" s="32" t="n">
+        <v>2546900</v>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Proforma vacancy/EGI figures as reported by each preparer (Ryan, Property Tax Advisors, or owner's analysis). 5970 Marion figures are from the owner's income-approach block in the 2024 P&amp;L workbook (PGI $172,800, 95% occ, NOI $159,938, 6.5% cap → $2,460,577; assigned $2,527,915).  Self-storage proformas (10350 Washington, 15413 E 18th, 1540 Altura) are Ryan LLC income-capitalization appeals valuing the 100% NNN-leased self-storage facility as a single blanket tenancy, not unit-level rent rolls. Altura Blvd doc header prints 'Assessment Year: 2026' but its own value table is labeled 2025 (reproduced as printed).</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n"/>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+      <c r="F28" s="20" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3631,7 +4328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3655,7 +4352,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3770,23 +4466,88 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Net = Total Income − Total Expense as printed. Bases differ: 5970 Marion &amp; Broadview totals include financing/depreciation, so they are cash-flow / tax figures, not NOI. TempTee reported operating expenses only. See 'Assessments &amp; Valuation' tab for stabilized NOI proformas.</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="21" t="n"/>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 proforma</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>676706</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>372188</v>
+      </c>
+      <c r="D9" s="32">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Ryan appeal income-cap proforma (EGI/non-reimb. exp.); no actual P&amp;L in source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>783123.25</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>499759.18</v>
+      </c>
+      <c r="D10" s="32">
+        <f>B10-C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>CubeSmart consolidated income statement, store 6730 (YTD through Dec 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>414633.83</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>328355.94</v>
+      </c>
+      <c r="D11" s="32">
+        <f>B11-C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>CubeSmart consolidated income statement, store 6731 (YTD through Dec 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Net = Total Income − Total Expense as printed. Bases differ: 5970 Marion &amp; Broadview totals include financing/depreciation, so they are cash-flow / tax figures, not NOI. TempTee reported operating expenses only. See 'Assessments &amp; Valuation' tab for stabilized NOI proformas. 10350 Washington's actual on-site P&amp;L was not included in its appeal package — only the income-cap proforma is available, so its 'income/expense' here are EGI and non-reimbursable opex from that proforma, not a real P&amp;L. The two Winner Storage/CubeSmart comps report true YTD actuals.</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3798,7 +4559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3822,7 +4583,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5207,6 +5967,825 @@
       <c r="E65" s="18" t="inlineStr">
         <is>
           <t>Printed total: $316,181.00. IRS Form 8825; net rental loss $(8,364). Tax basis (incl. depreciation, amortization &amp; interest).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="33" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 Proforma</t>
+        </is>
+      </c>
+      <c r="B66" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C66" s="33" t="inlineStr">
+        <is>
+          <t>Gross Potential Rent (Base Rent, NNN, $16.50/SF)</t>
+        </is>
+      </c>
+      <c r="D66" s="34" t="n">
+        <v>796125</v>
+      </c>
+      <c r="E66" s="33" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="33" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 Proforma</t>
+        </is>
+      </c>
+      <c r="B67" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C67" s="33" t="inlineStr">
+        <is>
+          <t>Less: Vacancy &amp; Credit Loss (15%)</t>
+        </is>
+      </c>
+      <c r="D67" s="34" t="n">
+        <v>-119419</v>
+      </c>
+      <c r="E67" s="33" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="33" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 Proforma</t>
+        </is>
+      </c>
+      <c r="B68" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C68" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL INCOME</t>
+        </is>
+      </c>
+      <c r="D68" s="34">
+        <f>SUM(D66:D67)</f>
+        <v/>
+      </c>
+      <c r="E68" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="33" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 Proforma</t>
+        </is>
+      </c>
+      <c r="B69" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C69" s="33" t="inlineStr">
+        <is>
+          <t>Non-Reimbursable Expenses (55% of EGI)</t>
+        </is>
+      </c>
+      <c r="D69" s="34" t="n">
+        <v>372188</v>
+      </c>
+      <c r="E69" s="33" t="inlineStr">
+        <is>
+          <t>Yields NOI $304,518 at 6.75% cap = $4,510,000 indicated value</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="33" t="inlineStr">
+        <is>
+          <t>10350 Washington St (R0040829) — 2026 Proforma</t>
+        </is>
+      </c>
+      <c r="B70" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C70" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSE</t>
+        </is>
+      </c>
+      <c r="D70" s="34">
+        <f>SUM(D69:D69)</f>
+        <v/>
+      </c>
+      <c r="E70" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C72" s="33" t="inlineStr">
+        <is>
+          <t>Net Rental Income</t>
+        </is>
+      </c>
+      <c r="D72" s="34" t="n">
+        <v>731252.08</v>
+      </c>
+      <c r="E72" s="33" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B73" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C73" s="33" t="inlineStr">
+        <is>
+          <t>Total Fees (admin/late/other, net of waivers &amp; chargebacks)</t>
+        </is>
+      </c>
+      <c r="D73" s="34" t="n">
+        <v>51871.17</v>
+      </c>
+      <c r="E73" s="33" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B74" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C74" s="33" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="D74" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="33" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B75" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C75" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL INCOME</t>
+        </is>
+      </c>
+      <c r="D75" s="34">
+        <f>SUM(D72:D74)</f>
+        <v/>
+      </c>
+      <c r="E75" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B76" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C76" s="33" t="inlineStr">
+        <is>
+          <t>Payroll Expense</t>
+        </is>
+      </c>
+      <c r="D76" s="34" t="n">
+        <v>84368.25</v>
+      </c>
+      <c r="E76" s="33" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B77" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C77" s="33" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D77" s="34" t="n">
+        <v>20743.13</v>
+      </c>
+      <c r="E77" s="33" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B78" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C78" s="33" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D78" s="34" t="n">
+        <v>17362.79</v>
+      </c>
+      <c r="E78" s="33" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B79" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C79" s="33" t="inlineStr">
+        <is>
+          <t>Other Controllable Expenses</t>
+        </is>
+      </c>
+      <c r="D79" s="34" t="n">
+        <v>48137.71</v>
+      </c>
+      <c r="E79" s="33" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B80" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C80" s="33" t="inlineStr">
+        <is>
+          <t>Marketing Expense</t>
+        </is>
+      </c>
+      <c r="D80" s="34" t="n">
+        <v>25974.66</v>
+      </c>
+      <c r="E80" s="33" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B81" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C81" s="33" t="inlineStr">
+        <is>
+          <t>Snow Removal &amp; Salting</t>
+        </is>
+      </c>
+      <c r="D81" s="34" t="n">
+        <v>3890</v>
+      </c>
+      <c r="E81" s="33" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B82" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C82" s="33" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="D82" s="34" t="n">
+        <v>350</v>
+      </c>
+      <c r="E82" s="33" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B83" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C83" s="33" t="inlineStr">
+        <is>
+          <t>Third-Party Management Fees</t>
+        </is>
+      </c>
+      <c r="D83" s="34" t="n">
+        <v>41598.27</v>
+      </c>
+      <c r="E83" s="33" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B84" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C84" s="33" t="inlineStr">
+        <is>
+          <t>Less: Other Income (Sales Tax Collection Allowance)</t>
+        </is>
+      </c>
+      <c r="D84" s="34" t="n">
+        <v>-14.31</v>
+      </c>
+      <c r="E84" s="33" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B85" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C85" s="33" t="inlineStr">
+        <is>
+          <t>Property Tax Expense (Gross Receipts Tax)</t>
+        </is>
+      </c>
+      <c r="D85" s="34" t="n">
+        <v>246826.26</v>
+      </c>
+      <c r="E85" s="33" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B86" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C86" s="33" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="D86" s="34" t="n">
+        <v>10522.42</v>
+      </c>
+      <c r="E86" s="33" t="inlineStr">
+        <is>
+          <t>CubeSmart consolidated income statement, store 6730</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="33" t="inlineStr">
+        <is>
+          <t>15413 E 18th Ave (R0086010) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B87" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C87" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSE</t>
+        </is>
+      </c>
+      <c r="D87" s="34">
+        <f>SUM(D76:D86)</f>
+        <v/>
+      </c>
+      <c r="E87" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B89" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C89" s="33" t="inlineStr">
+        <is>
+          <t>Net Rental Income</t>
+        </is>
+      </c>
+      <c r="D89" s="34" t="n">
+        <v>383165.98</v>
+      </c>
+      <c r="E89" s="33" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C90" s="33" t="inlineStr">
+        <is>
+          <t>Total Fees (admin/late/other, net of waivers &amp; chargebacks)</t>
+        </is>
+      </c>
+      <c r="D90" s="34" t="n">
+        <v>31467.84</v>
+      </c>
+      <c r="E90" s="33" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B91" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C91" s="33" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="D91" s="34" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E91" s="33" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B92" s="33" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C92" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL INCOME</t>
+        </is>
+      </c>
+      <c r="D92" s="34">
+        <f>SUM(D89:D91)</f>
+        <v/>
+      </c>
+      <c r="E92" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B93" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C93" s="33" t="inlineStr">
+        <is>
+          <t>Payroll Expense</t>
+        </is>
+      </c>
+      <c r="D93" s="34" t="n">
+        <v>69477.36</v>
+      </c>
+      <c r="E93" s="33" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B94" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C94" s="33" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D94" s="34" t="n">
+        <v>15848.82</v>
+      </c>
+      <c r="E94" s="33" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B95" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C95" s="33" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D95" s="34" t="n">
+        <v>25497.14</v>
+      </c>
+      <c r="E95" s="33" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B96" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C96" s="33" t="inlineStr">
+        <is>
+          <t>Other Controllable Expenses</t>
+        </is>
+      </c>
+      <c r="D96" s="34" t="n">
+        <v>40436.57</v>
+      </c>
+      <c r="E96" s="33" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B97" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C97" s="33" t="inlineStr">
+        <is>
+          <t>Marketing Expense</t>
+        </is>
+      </c>
+      <c r="D97" s="34" t="n">
+        <v>24474.39</v>
+      </c>
+      <c r="E97" s="33" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B98" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C98" s="33" t="inlineStr">
+        <is>
+          <t>Snow Removal &amp; Salting</t>
+        </is>
+      </c>
+      <c r="D98" s="34" t="n">
+        <v>2180</v>
+      </c>
+      <c r="E98" s="33" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B99" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C99" s="33" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="D99" s="34" t="n">
+        <v>350</v>
+      </c>
+      <c r="E99" s="33" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B100" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C100" s="33" t="inlineStr">
+        <is>
+          <t>Third-Party Management Fees</t>
+        </is>
+      </c>
+      <c r="D100" s="34" t="n">
+        <v>22457.4</v>
+      </c>
+      <c r="E100" s="33" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B101" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C101" s="33" t="inlineStr">
+        <is>
+          <t>Less: Other Income (Sales Tax Collection Allowance)</t>
+        </is>
+      </c>
+      <c r="D101" s="34" t="n">
+        <v>-12.01</v>
+      </c>
+      <c r="E101" s="33" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B102" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C102" s="33" t="inlineStr">
+        <is>
+          <t>Property Tax Expense (Gross Receipts Tax)</t>
+        </is>
+      </c>
+      <c r="D102" s="34" t="n">
+        <v>121803.84</v>
+      </c>
+      <c r="E102" s="33" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B103" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C103" s="33" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="D103" s="34" t="n">
+        <v>5842.43</v>
+      </c>
+      <c r="E103" s="33" t="inlineStr">
+        <is>
+          <t>CubeSmart consolidated income statement, store 6731</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="33" t="inlineStr">
+        <is>
+          <t>1540 Altura Blvd (R0085571) — Actual Dec 2024 YTD</t>
+        </is>
+      </c>
+      <c r="B104" s="33" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C104" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSE</t>
+        </is>
+      </c>
+      <c r="D104" s="34">
+        <f>SUM(D93:D103)</f>
+        <v/>
+      </c>
+      <c r="E104" s="33" t="inlineStr">
+        <is>
+          <t>Printed total.</t>
         </is>
       </c>
     </row>
@@ -5249,7 +6828,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5385,7 +6963,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
@@ -5405,4 +6982,750 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>SELF-STORAGE INCOME &amp; EXPENSE COMPARISON — DECEMBER HEARINGS</t>
+        </is>
+      </c>
+      <c r="B1" s="36" t="n"/>
+      <c r="C1" s="36" t="n"/>
+      <c r="D1" s="36" t="n"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="37" t="inlineStr">
+        <is>
+          <t>Subject: 10350 Washington Street (R0040829) vs. comparable Adams County self-storage appeals in the same folder  |  Updated 2026-08-19</t>
+        </is>
+      </c>
+      <c r="B2" s="36" t="n"/>
+      <c r="C2" s="36" t="n"/>
+      <c r="D2" s="36" t="n"/>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="38" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SUBJECT
+10350 Washington St
+(R0040829)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>COMP 1
+15413 E 18th Ave, Aurora
+(R0086010)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>COMP 2
+1540 Altura Blvd, Aurora
+(R0085571)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>PROPERTY PROFILE</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n"/>
+      <c r="C5" s="40" t="n"/>
+      <c r="D5" s="40" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>Owner / Client</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>DSI Special Situations Fund B</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC / PTA USI No 730</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>Winner Storage LLC / PTA USI No 731</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>Parcel Number</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>0171914201013</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>0182132318001</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>0182131405022</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Year Built</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="n">
+        <v>1985</v>
+      </c>
+      <c r="C8" s="43" t="n">
+        <v>1984</v>
+      </c>
+      <c r="D8" s="43" t="n">
+        <v>1978</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Net Leasable Area (SF)</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="n">
+        <v>48250</v>
+      </c>
+      <c r="C9" s="45" t="n">
+        <v>57742</v>
+      </c>
+      <c r="D9" s="45" t="n">
+        <v>27139</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>Site Area (Acres)</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C10" s="47" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="D10" s="47" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>Occupancy (Jun 2024, per appeal)</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>84% actual / 85% stabilized</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>87% actual / 88% stabilized</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>0% vacancy assumed in proforma</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>ASSESSED VALUE</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n"/>
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="40" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Assessor's Value</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="n">
+        <v>5428808</v>
+      </c>
+      <c r="C13" s="49" t="n">
+        <v>8187500</v>
+      </c>
+      <c r="D13" s="49" t="n">
+        <v>3309468</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Value per SF</t>
+        </is>
+      </c>
+      <c r="B14" s="50" t="n">
+        <v>112.5141554404145</v>
+      </c>
+      <c r="C14" s="51" t="n">
+        <v>141.7945343077829</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>121.9450974612182</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Taxpayer's Opinion of Value</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="n">
+        <v>4510000</v>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>6610000</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>2546900</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Opinion per SF</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="n">
+        <v>93.47150259067358</v>
+      </c>
+      <c r="C16" s="51" t="n">
+        <v>114.4747324304666</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>93.84649397545967</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Assessment / Tax Year</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D17" s="43" t="inlineStr">
+        <is>
+          <t>2025 (per value table; header says 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>INCOME-APPROACH PROFORMA (Ryan LLC appeal — all three)</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n"/>
+      <c r="C18" s="40" t="n"/>
+      <c r="D18" s="40" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>Gross Potential Rent</t>
+        </is>
+      </c>
+      <c r="B19" s="48" t="n">
+        <v>796125</v>
+      </c>
+      <c r="C19" s="49" t="n">
+        <v>750646</v>
+      </c>
+      <c r="D19" s="49" t="n">
+        <v>413870</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Base Rent per SF</t>
+        </is>
+      </c>
+      <c r="B20" s="50" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C20" s="51" t="n">
+        <v>13</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>Vacancy &amp; Credit Loss</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>15% / $119,419</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="inlineStr">
+        <is>
+          <t>12% / $90,078</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="inlineStr">
+        <is>
+          <t>0% / $0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>Effective Gross Income (EGI)</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="n">
+        <v>676706</v>
+      </c>
+      <c r="C22" s="49" t="n">
+        <v>660568</v>
+      </c>
+      <c r="D22" s="49" t="n">
+        <v>413870</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>Operating / Non-Reimbursable Expenses</t>
+        </is>
+      </c>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>55% EGI / $372,188</t>
+        </is>
+      </c>
+      <c r="C23" s="43" t="inlineStr">
+        <is>
+          <t>35% EGI / $231,199</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
+        <is>
+          <t>60% EGI / $248,322</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>Net Operating Income (NOI)</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="n">
+        <v>304518</v>
+      </c>
+      <c r="C24" s="54" t="n">
+        <v>429370</v>
+      </c>
+      <c r="D24" s="54" t="n">
+        <v>165548</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>NOI per SF</t>
+        </is>
+      </c>
+      <c r="B25" s="50" t="n">
+        <v>6.311253886010363</v>
+      </c>
+      <c r="C25" s="51" t="n">
+        <v>7.436008451387205</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <v>6.100003684734147</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>Cap Rate</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="C26" s="56" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="D26" s="56" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="52" t="inlineStr">
+        <is>
+          <t>Indicated Value (Income Approach)</t>
+        </is>
+      </c>
+      <c r="B27" s="53" t="n">
+        <v>4510000</v>
+      </c>
+      <c r="C27" s="54" t="n">
+        <v>6610000</v>
+      </c>
+      <c r="D27" s="54" t="n">
+        <v>2546900</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>ACTUAL OPERATING STATEMENT — Dec 2024 YTD (CubeSmart-managed comps only)</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="n"/>
+      <c r="C28" s="40" t="n"/>
+      <c r="D28" s="40" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>Net Rental Income</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C29" s="49" t="n">
+        <v>731252.08</v>
+      </c>
+      <c r="D29" s="49" t="n">
+        <v>383165.98</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>Fees &amp; Other Income</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C30" s="49" t="n">
+        <v>51871.17</v>
+      </c>
+      <c r="D30" s="49" t="n">
+        <v>31467.85</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="52" t="inlineStr">
+        <is>
+          <t>TOTAL ACTUAL INCOME</t>
+        </is>
+      </c>
+      <c r="B31" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C31" s="54" t="n">
+        <v>783123.25</v>
+      </c>
+      <c r="D31" s="54" t="n">
+        <v>414633.83</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>Payroll Expense</t>
+        </is>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C32" s="49" t="n">
+        <v>84368.25</v>
+      </c>
+      <c r="D32" s="49" t="n">
+        <v>69477.36</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="41" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B33" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="n">
+        <v>20743.13</v>
+      </c>
+      <c r="D33" s="49" t="n">
+        <v>15848.82</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C34" s="49" t="n">
+        <v>17362.79</v>
+      </c>
+      <c r="D34" s="49" t="n">
+        <v>25497.14</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B35" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" s="49" t="n">
+        <v>25974.66</v>
+      </c>
+      <c r="D35" s="49" t="n">
+        <v>24474.39</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>Other Controllable Expenses</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C36" s="49" t="n">
+        <v>48137.71</v>
+      </c>
+      <c r="D36" s="49" t="n">
+        <v>40436.57</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>Property Tax (Gross Receipts Tax)</t>
+        </is>
+      </c>
+      <c r="B37" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C37" s="49" t="n">
+        <v>246826.26</v>
+      </c>
+      <c r="D37" s="49" t="n">
+        <v>121803.84</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" s="49" t="n">
+        <v>10522.42</v>
+      </c>
+      <c r="D38" s="49" t="n">
+        <v>5842.43</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>Mgmt Fee, Snow Removal, Prof. Fees (net)</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="n">
+        <v>45823.96</v>
+      </c>
+      <c r="D39" s="49" t="n">
+        <v>24975.39</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="52" t="inlineStr">
+        <is>
+          <t>TOTAL ACTUAL EXPENSE</t>
+        </is>
+      </c>
+      <c r="B40" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" s="54" t="n">
+        <v>499759.18</v>
+      </c>
+      <c r="D40" s="54" t="n">
+        <v>328355.94</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="52" t="inlineStr">
+        <is>
+          <t>ACTUAL NET OPERATING INCOME</t>
+        </is>
+      </c>
+      <c r="B41" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C41" s="54" t="n">
+        <v>283364.07</v>
+      </c>
+      <c r="D41" s="54" t="n">
+        <v>86277.89</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>Actual NOI per SF</t>
+        </is>
+      </c>
+      <c r="B42" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C42" s="51" t="n">
+        <v>4.907416958193343</v>
+      </c>
+      <c r="D42" s="51" t="n">
+        <v>3.179110873650466</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>Actual Expense Ratio (Exp / Total Income)</t>
+        </is>
+      </c>
+      <c r="B43" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C43" s="56" t="n">
+        <v>0.6381615920610197</v>
+      </c>
+      <c r="D43" s="56" t="n">
+        <v>0.7919178712455759</v>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="58" t="inlineStr">
+        <is>
+          <t>Notes: All three properties are Adams County self-storage tax appeals prepared by Ryan LLC (Declan Fassig), valued as of 6/30/2024, from the 'R0040829 - 10350 Washington Street' folder under December Hearings. Proforma figures (income-approach appeal) are apples-to-apples across all three. Actual operating statements are only available for the two Winner Storage/CubeSmart comps (15413 E 18th Ave and 1540 Altura Blvd) — 10350 Washington's appeal package did not include an actual P&amp;L, only the income-cap proforma, so its actual-statement cells are marked '—'. 1540 Altura Blvd's header prints 'Assessment Year: 2026' but its own value table and income statement are labeled 2025 — reproduced as printed. Full line-item detail and source citations are in the 'Assessments &amp; Valuation' and 'Income-Expense Detail' tabs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:D28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Expense Comps ($/SF) tab organized by OCC code and size
New "Expense Comps ($ per SF)" tab breaks out Insurance, Utilities,
CAM+Repairs & Maintenance, and Management on a per-SF basis for every
property with actual expense data, sorted/filterable by an inferred
OCC Code and building Size (SF) for comp-building. NNN leases (Amazon
x3, Home Depot) are listed separately as excluded since the tenant
pays these costs directly.

Also re-derives full GL-account expense detail (previously only
summary totals) for 6 Majestic Commercenter buildings, each verified
to the cent against the printed Total Operating Expenses.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SUHi3FURZTyT771xGP7HPj
</commit_message>
<xml_diff>
--- a/Master_Property_Database.xlsx
+++ b/Master_Property_Database.xlsx
@@ -13,23 +13,27 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments &amp; Valuation" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expense Comps ($ per SF)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Expense Comps ($ per SF)'!$A$4:$Q$22</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.###"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);-"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="168" formatCode="$0.00"/>
+    <numFmt numFmtId="169" formatCode="$0.00;($0.00);&quot;n/a&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +84,11 @@
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="8">
@@ -190,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -295,6 +304,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -14991,6 +15018,1511 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>EXPENSE COMPS — $ PER SQUARE FOOT</t>
+        </is>
+      </c>
+      <c r="B1" s="47" t="n"/>
+      <c r="C1" s="47" t="n"/>
+      <c r="D1" s="47" t="n"/>
+      <c r="E1" s="47" t="n"/>
+      <c r="F1" s="47" t="n"/>
+      <c r="G1" s="47" t="n"/>
+      <c r="H1" s="47" t="n"/>
+      <c r="I1" s="47" t="n"/>
+      <c r="J1" s="47" t="n"/>
+      <c r="K1" s="47" t="n"/>
+      <c r="L1" s="47" t="n"/>
+      <c r="M1" s="47" t="n"/>
+      <c r="N1" s="47" t="n"/>
+      <c r="O1" s="47" t="n"/>
+      <c r="P1" s="47" t="n"/>
+      <c r="Q1" s="47" t="n"/>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>Insurance, Utilities, CAM+Repairs &amp; Maintenance, and Management costs per SF — organize/filter by OCC Code and Size (SF) to build comp sets</t>
+        </is>
+      </c>
+      <c r="B2" s="47" t="n"/>
+      <c r="C2" s="47" t="n"/>
+      <c r="D2" s="47" t="n"/>
+      <c r="E2" s="47" t="n"/>
+      <c r="F2" s="47" t="n"/>
+      <c r="G2" s="47" t="n"/>
+      <c r="H2" s="47" t="n"/>
+      <c r="I2" s="47" t="n"/>
+      <c r="J2" s="47" t="n"/>
+      <c r="K2" s="47" t="n"/>
+      <c r="L2" s="47" t="n"/>
+      <c r="M2" s="47" t="n"/>
+      <c r="N2" s="47" t="n"/>
+      <c r="O2" s="47" t="n"/>
+      <c r="P2" s="47" t="n"/>
+      <c r="Q2" s="47" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="49" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>OCC Code</t>
+        </is>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>Property Type / Use</t>
+        </is>
+      </c>
+      <c r="D4" s="49" t="inlineStr">
+        <is>
+          <t>Size (SF)</t>
+        </is>
+      </c>
+      <c r="E4" s="49" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="F4" s="49" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="G4" s="49" t="inlineStr">
+        <is>
+          <t>Occupancy</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
+        <is>
+          <t>Insurance $</t>
+        </is>
+      </c>
+      <c r="I4" s="49" t="inlineStr">
+        <is>
+          <t>Insurance $/SF</t>
+        </is>
+      </c>
+      <c r="J4" s="49" t="inlineStr">
+        <is>
+          <t>Utilities $</t>
+        </is>
+      </c>
+      <c r="K4" s="49" t="inlineStr">
+        <is>
+          <t>Utilities $/SF</t>
+        </is>
+      </c>
+      <c r="L4" s="49" t="inlineStr">
+        <is>
+          <t>CAM + R&amp;M $</t>
+        </is>
+      </c>
+      <c r="M4" s="49" t="inlineStr">
+        <is>
+          <t>CAM + R&amp;M $/SF</t>
+        </is>
+      </c>
+      <c r="N4" s="49" t="inlineStr">
+        <is>
+          <t>Management $</t>
+        </is>
+      </c>
+      <c r="O4" s="49" t="inlineStr">
+        <is>
+          <t>Management $/SF</t>
+        </is>
+      </c>
+      <c r="P4" s="49" t="inlineStr">
+        <is>
+          <t>Total (4 cats) $/SF</t>
+        </is>
+      </c>
+      <c r="Q4" s="49" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>125 Bridge St (Broadview)</t>
+        </is>
+      </c>
+      <c r="B5" s="50" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>Commercial (multi-tenant industrial)</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>2024 (IRS Form 8825)</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>Mostly leased (1-2 units vacant)</t>
+        </is>
+      </c>
+      <c r="H5" s="40" t="n">
+        <v>12004</v>
+      </c>
+      <c r="J5" s="40" t="n">
+        <v>4731</v>
+      </c>
+      <c r="L5" s="40" t="n">
+        <v>100279</v>
+      </c>
+      <c r="N5" s="33" t="n"/>
+      <c r="Q5" s="52" t="inlineStr">
+        <is>
+          <t>CAM/R&amp;M = 'Repairs' line per Form 8825. No separate management-fee line on the tax return (bundled in 'Other $39,767' or self-managed). Building SF not captured in Property Master (multi-suite building; unit-level rents only) — $/SF not computable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>2780 N. Tower Road</t>
+        </is>
+      </c>
+      <c r="B6" s="50" t="inlineStr">
+        <is>
+          <t>IND-DIST</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Distribution (single tenant)</t>
+        </is>
+      </c>
+      <c r="D6" s="53" t="n">
+        <v>386000</v>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>Actual (NNN — tenant-paid)</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>100% (single tenant)</t>
+        </is>
+      </c>
+      <c r="H6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="54">
+        <f>H6/D6</f>
+        <v/>
+      </c>
+      <c r="J6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="54">
+        <f>J6/D6</f>
+        <v/>
+      </c>
+      <c r="L6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="54">
+        <f>L6/D6</f>
+        <v/>
+      </c>
+      <c r="N6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="54">
+        <f>N6/D6</f>
+        <v/>
+      </c>
+      <c r="P6" s="55">
+        <f>SUM(H6,J6,L6,N6)/D6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="52" t="inlineStr">
+        <is>
+          <t>Landlord P&amp;L has NO Insurance/Utilities/CAM/Management GL lines — this is a true NNN lease where the tenant pays all operating costs directly. Landlord-side costs are limited to G&amp;A (bank fees, legal, accounting), interest, and depreciation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>2780 N. Tower Road</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>IND-DIST</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Distribution (single tenant)</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="n">
+        <v>386000</v>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>Actual (NNN — tenant-paid)</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>100% (single tenant)</t>
+        </is>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="54">
+        <f>H7/D7</f>
+        <v/>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>687</v>
+      </c>
+      <c r="K7" s="54">
+        <f>J7/D7</f>
+        <v/>
+      </c>
+      <c r="L7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="54">
+        <f>L7/D7</f>
+        <v/>
+      </c>
+      <c r="N7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="54">
+        <f>N7/D7</f>
+        <v/>
+      </c>
+      <c r="P7" s="55">
+        <f>SUM(H7,J7,L7,N7)/D7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="52" t="inlineStr">
+        <is>
+          <t>Same NNN structure as FY2024; $687 utilities appears to be a minor landlord-side true-up, not a recurring cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2011 E 58th Ave (TempTee)</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Mfg / Food Processing</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="n">
+        <v>17000</v>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>2024 survey (Oct'23-Sep'24)</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>100% Owner-Occupied</t>
+        </is>
+      </c>
+      <c r="H8" s="40" t="n">
+        <v>14050</v>
+      </c>
+      <c r="I8" s="54">
+        <f>H8/D8</f>
+        <v/>
+      </c>
+      <c r="J8" s="40" t="n">
+        <v>102000</v>
+      </c>
+      <c r="K8" s="54">
+        <f>J8/D8</f>
+        <v/>
+      </c>
+      <c r="L8" s="40" t="n">
+        <v>22000</v>
+      </c>
+      <c r="M8" s="54">
+        <f>L8/D8</f>
+        <v/>
+      </c>
+      <c r="N8" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="54">
+        <f>N8/D8</f>
+        <v/>
+      </c>
+      <c r="P8" s="55">
+        <f>SUM(H8,J8,L8,N8)/D8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="52" t="inlineStr">
+        <is>
+          <t>CAM/R&amp;M = Building R&amp;M $10,000 + Snow/Trash Removal $12,000. Ground Maintenance &amp; Janitorial reported 'in house' = $0 (not truly zero cost, just unreported/self-performed). No 3rd-party management fee (owner-occupied).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>TrusTile Doors</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Manufacturing (doors)</t>
+        </is>
+      </c>
+      <c r="D9" s="51" t="n"/>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>Oct'23-Sep'24 survey</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>100% Owner-Occupied</t>
+        </is>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>361160</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>1031487</v>
+      </c>
+      <c r="L9" s="40" t="n">
+        <v>1695350</v>
+      </c>
+      <c r="N9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="52" t="inlineStr">
+        <is>
+          <t>CAM/R&amp;M = Building R&amp;M $796,122 + Janitorial $150,032 + Snow/Trash Removal $749,196. No management fee (owner-occupied, no leasing). Building SF not stated on the county survey form — $/SF not computable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>5970 Marion Drive</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - 2-unit</t>
+        </is>
+      </c>
+      <c r="D10" s="53" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>100% (2 units)</t>
+        </is>
+      </c>
+      <c r="H10" s="40" t="n">
+        <v>10241.26</v>
+      </c>
+      <c r="I10" s="54">
+        <f>H10/D10</f>
+        <v/>
+      </c>
+      <c r="J10" s="40" t="n">
+        <v>2569.85</v>
+      </c>
+      <c r="K10" s="54">
+        <f>J10/D10</f>
+        <v/>
+      </c>
+      <c r="L10" s="40" t="n">
+        <v>1227.47</v>
+      </c>
+      <c r="M10" s="54">
+        <f>L10/D10</f>
+        <v/>
+      </c>
+      <c r="N10" s="40" t="n">
+        <v>6000</v>
+      </c>
+      <c r="O10" s="54">
+        <f>N10/D10</f>
+        <v/>
+      </c>
+      <c r="P10" s="55">
+        <f>SUM(H10,J10,L10,N10)/D10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="52" t="inlineStr">
+        <is>
+          <t>Utilities = Water $2,175.55 + Sewer $394.30. CAM/R&amp;M = Inspection &amp; Compliance $100 + Snow Removal $927.47 + Common Area Clean $200. Mgmt: Deerwoods Management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>5970 Marion Drive</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - 2-unit</t>
+        </is>
+      </c>
+      <c r="D11" s="53" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>100% (2 units)</t>
+        </is>
+      </c>
+      <c r="H11" s="40" t="n">
+        <v>8640.99</v>
+      </c>
+      <c r="I11" s="54">
+        <f>H11/D11</f>
+        <v/>
+      </c>
+      <c r="J11" s="40" t="n">
+        <v>2308.09</v>
+      </c>
+      <c r="K11" s="54">
+        <f>J11/D11</f>
+        <v/>
+      </c>
+      <c r="L11" s="40" t="n">
+        <v>50376.31</v>
+      </c>
+      <c r="M11" s="54">
+        <f>L11/D11</f>
+        <v/>
+      </c>
+      <c r="N11" s="40" t="n">
+        <v>6000</v>
+      </c>
+      <c r="O11" s="54">
+        <f>N11/D11</f>
+        <v/>
+      </c>
+      <c r="P11" s="55">
+        <f>SUM(H11,J11,L11,N11)/D11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="52" t="inlineStr">
+        <is>
+          <t>Utilities = Water $2,157.08 + Trash $151.01. CAM/R&amp;M = Electrical Repairs &amp; Lighting $1,550 + Roofing Repairs $47,000 (one-off) + Drywall Repairs $810 + Snow Removal $1,016.31 + Inspection &amp; Compliance $110 — large roof repair skews this year high.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 26</t>
+        </is>
+      </c>
+      <c r="B12" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D12" s="53" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>100% (single tenant)</t>
+        </is>
+      </c>
+      <c r="H12" s="40" t="n">
+        <v>30594</v>
+      </c>
+      <c r="I12" s="54">
+        <f>H12/D12</f>
+        <v/>
+      </c>
+      <c r="J12" s="40" t="n">
+        <v>477.83</v>
+      </c>
+      <c r="K12" s="54">
+        <f>J12/D12</f>
+        <v/>
+      </c>
+      <c r="L12" s="40" t="n">
+        <v>95782.41</v>
+      </c>
+      <c r="M12" s="54">
+        <f>L12/D12</f>
+        <v/>
+      </c>
+      <c r="N12" s="40" t="n">
+        <v>36084.88</v>
+      </c>
+      <c r="O12" s="54">
+        <f>N12/D12</f>
+        <v/>
+      </c>
+      <c r="P12" s="55">
+        <f>SUM(H12,J12,L12,N12)/D12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="52" t="inlineStr">
+        <is>
+          <t>Utilities landlord-side captured only 'Fire Service' — single-tenant NNN, tenant pays electricity/gas/water directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 22</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D13" s="53" t="n">
+        <v>200090</v>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="H13" s="40" t="n">
+        <v>26308</v>
+      </c>
+      <c r="I13" s="54">
+        <f>H13/D13</f>
+        <v/>
+      </c>
+      <c r="J13" s="40" t="n">
+        <v>72124.12</v>
+      </c>
+      <c r="K13" s="54">
+        <f>J13/D13</f>
+        <v/>
+      </c>
+      <c r="L13" s="40" t="n">
+        <v>149100.03</v>
+      </c>
+      <c r="M13" s="54">
+        <f>L13/D13</f>
+        <v/>
+      </c>
+      <c r="N13" s="40" t="n">
+        <v>48882.34</v>
+      </c>
+      <c r="O13" s="54">
+        <f>N13/D13</f>
+        <v/>
+      </c>
+      <c r="P13" s="55">
+        <f>SUM(H13,J13,L13,N13)/D13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="52" t="inlineStr">
+        <is>
+          <t>Only building in this batch with partial (75%) actual occupancy at DOV. GL carries two account series (5xxx and 6xxx) suggesting two building sections; both rolled together here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Broadway Logistics Center</t>
+        </is>
+      </c>
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D14" s="53" t="n">
+        <v>201025</v>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>0% (100% vacant)</t>
+        </is>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>32411.18</v>
+      </c>
+      <c r="I14" s="54">
+        <f>H14/D14</f>
+        <v/>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>11508.48</v>
+      </c>
+      <c r="K14" s="54">
+        <f>J14/D14</f>
+        <v/>
+      </c>
+      <c r="L14" s="40" t="n">
+        <v>9383.52</v>
+      </c>
+      <c r="M14" s="54">
+        <f>L14/D14</f>
+        <v/>
+      </c>
+      <c r="N14" s="40" t="n">
+        <v>12500</v>
+      </c>
+      <c r="O14" s="54">
+        <f>N14/D14</f>
+        <v/>
+      </c>
+      <c r="P14" s="55">
+        <f>SUM(H14,J14,L14,N14)/D14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="52" t="inlineStr">
+        <is>
+          <t>Utilities = Recoverable $11,084.46 + Non-Recoverable 'Electricity Vacant' $424.02. CAM/R&amp;M = Repair &amp; Maint $3,639.29 + Contract Services (Fire Alarm/Sweeping/Janitorial) $5,744.23. Building 100% vacant all year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 24</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D15" s="53" t="n">
+        <v>215030</v>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>100% (multi-tenant)</t>
+        </is>
+      </c>
+      <c r="H15" s="40" t="n">
+        <v>30832</v>
+      </c>
+      <c r="I15" s="54">
+        <f>H15/D15</f>
+        <v/>
+      </c>
+      <c r="J15" s="40" t="n">
+        <v>101924.33</v>
+      </c>
+      <c r="K15" s="54">
+        <f>J15/D15</f>
+        <v/>
+      </c>
+      <c r="L15" s="40" t="n">
+        <v>127450.06</v>
+      </c>
+      <c r="M15" s="54">
+        <f>L15/D15</f>
+        <v/>
+      </c>
+      <c r="N15" s="40" t="n">
+        <v>71320.8</v>
+      </c>
+      <c r="O15" s="54">
+        <f>N15/D15</f>
+        <v/>
+      </c>
+      <c r="P15" s="55">
+        <f>SUM(H15,J15,L15,N15)/D15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="52" t="inlineStr">
+        <is>
+          <t>Full electricity/gas/water utilities present (multi-tenant, landlord pays and recovers via CAM). CAM/R&amp;M includes a '5312 Other-DTR' pass-through line ($5,821.17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 11</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D16" s="53" t="n">
+        <v>244920</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="inlineStr">
+        <is>
+          <t>0% (100% vacant)</t>
+        </is>
+      </c>
+      <c r="H16" s="40" t="n">
+        <v>9460.52</v>
+      </c>
+      <c r="I16" s="54">
+        <f>H16/D16</f>
+        <v/>
+      </c>
+      <c r="J16" s="40" t="n">
+        <v>67358.14999999999</v>
+      </c>
+      <c r="K16" s="54">
+        <f>J16/D16</f>
+        <v/>
+      </c>
+      <c r="L16" s="40" t="n">
+        <v>43289.06</v>
+      </c>
+      <c r="M16" s="54">
+        <f>L16/D16</f>
+        <v/>
+      </c>
+      <c r="N16" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="54">
+        <f>N16/D16</f>
+        <v/>
+      </c>
+      <c r="P16" s="55">
+        <f>SUM(H16,J16,L16,N16)/D16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="52" t="inlineStr">
+        <is>
+          <t>Self-managed by Majestic Realty — no 3rd-party management-fee GL line. Building 100% vacant all year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Shamrock Foods</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="D17" s="53" t="n">
+        <v>329903</v>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>TY2025 appeal</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>Proforma Assumption (not actual — owner-occupied, no tenant)</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>100% Owner-Occupied</t>
+        </is>
+      </c>
+      <c r="H17" s="40" t="n">
+        <v>56908</v>
+      </c>
+      <c r="I17" s="54">
+        <f>H17/D17</f>
+        <v/>
+      </c>
+      <c r="J17" s="33" t="n"/>
+      <c r="L17" s="33" t="n"/>
+      <c r="N17" s="40" t="n">
+        <v>56908</v>
+      </c>
+      <c r="O17" s="54">
+        <f>N17/D17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="52" t="inlineStr">
+        <is>
+          <t>Insurance &amp; Management are the appeal's hypothetical fee-simple pro forma assumptions (3% of EGI each). Utilities and CAM/R&amp;M were not broken out separately — folded into the pro forma's blanket operating-expense load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>22100 E 26th Ave (ASB)</t>
+        </is>
+      </c>
+      <c r="B18" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="D18" s="53" t="n">
+        <v>406959</v>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>28% (6/30/2024)</t>
+        </is>
+      </c>
+      <c r="H18" s="40" t="n">
+        <v>201387.56</v>
+      </c>
+      <c r="I18" s="54">
+        <f>H18/D18</f>
+        <v/>
+      </c>
+      <c r="J18" s="40" t="n">
+        <v>124809.5</v>
+      </c>
+      <c r="K18" s="54">
+        <f>J18/D18</f>
+        <v/>
+      </c>
+      <c r="L18" s="40" t="n">
+        <v>97166.52</v>
+      </c>
+      <c r="M18" s="54">
+        <f>L18/D18</f>
+        <v/>
+      </c>
+      <c r="N18" s="40" t="n">
+        <v>36000</v>
+      </c>
+      <c r="O18" s="54">
+        <f>N18/D18</f>
+        <v/>
+      </c>
+      <c r="P18" s="55">
+        <f>SUM(H18,J18,L18,N18)/D18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="52" t="inlineStr">
+        <is>
+          <t>CAM/R&amp;M = Cleaning $2,250 + Repairs &amp; Maintenance $17,250 + Roads &amp; Grounds $49,573.29 + Security &amp; Life Safety $28,093.23. Monthly-column OCR on this statement was unreliable (already flagged in Income-Expense Detail); these are the clean category-level annual TOTAL lines, which do not net perfectly to the statement's overall Total Operating Expense due to that OCR issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>22100 E 26th Ave (ASB)</t>
+        </is>
+      </c>
+      <c r="B19" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="D19" s="53" t="n">
+        <v>406959</v>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>~22% (largely vacant, pre-Vederra lease)</t>
+        </is>
+      </c>
+      <c r="H19" s="40" t="n">
+        <v>140115.36</v>
+      </c>
+      <c r="I19" s="54">
+        <f>H19/D19</f>
+        <v/>
+      </c>
+      <c r="J19" s="40" t="n">
+        <v>200928.77</v>
+      </c>
+      <c r="K19" s="54">
+        <f>J19/D19</f>
+        <v/>
+      </c>
+      <c r="L19" s="40" t="n">
+        <v>58649.22</v>
+      </c>
+      <c r="M19" s="54">
+        <f>L19/D19</f>
+        <v/>
+      </c>
+      <c r="N19" s="40" t="n">
+        <v>36000</v>
+      </c>
+      <c r="O19" s="54">
+        <f>N19/D19</f>
+        <v/>
+      </c>
+      <c r="P19" s="55">
+        <f>SUM(H19,J19,L19,N19)/D19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="52" t="inlineStr">
+        <is>
+          <t>CAM/R&amp;M = Cleaning $3,480 + Repairs &amp; Maintenance $21,396.45 + Roads &amp; Grounds $25,320.33 + Security &amp; Life Safety $8,452.44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 29</t>
+        </is>
+      </c>
+      <c r="B20" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D20" s="53" t="n">
+        <v>452400</v>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F20" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="inlineStr">
+        <is>
+          <t>100% (multi-tenant)</t>
+        </is>
+      </c>
+      <c r="H20" s="40" t="n">
+        <v>69076</v>
+      </c>
+      <c r="I20" s="54">
+        <f>H20/D20</f>
+        <v/>
+      </c>
+      <c r="J20" s="40" t="n">
+        <v>1080.84</v>
+      </c>
+      <c r="K20" s="54">
+        <f>J20/D20</f>
+        <v/>
+      </c>
+      <c r="L20" s="40" t="n">
+        <v>170658.68</v>
+      </c>
+      <c r="M20" s="54">
+        <f>L20/D20</f>
+        <v/>
+      </c>
+      <c r="N20" s="40" t="n">
+        <v>123809.45</v>
+      </c>
+      <c r="O20" s="54">
+        <f>N20/D20</f>
+        <v/>
+      </c>
+      <c r="P20" s="55">
+        <f>SUM(H20,J20,L20,N20)/D20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="52" t="inlineStr">
+        <is>
+          <t>Utilities landlord-side captured only 'Fire Service' ($1,080.84) — electricity/gas/water appear tenant-billed direct or routed through a '5312 Other-DTR' pass-through account ($118,064.60, not classified into the 4 categories here). CAM/R&amp;M includes an unusually large $94,602 'Painting' line item (reproduced as printed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 12</t>
+        </is>
+      </c>
+      <c r="B21" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D21" s="53" t="n">
+        <v>461580</v>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>0% (100% vacant)</t>
+        </is>
+      </c>
+      <c r="H21" s="40" t="n">
+        <v>16527.93</v>
+      </c>
+      <c r="I21" s="54">
+        <f>H21/D21</f>
+        <v/>
+      </c>
+      <c r="J21" s="40" t="n">
+        <v>20820.4</v>
+      </c>
+      <c r="K21" s="54">
+        <f>J21/D21</f>
+        <v/>
+      </c>
+      <c r="L21" s="40" t="n">
+        <v>42752.71</v>
+      </c>
+      <c r="M21" s="54">
+        <f>L21/D21</f>
+        <v/>
+      </c>
+      <c r="N21" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="54">
+        <f>N21/D21</f>
+        <v/>
+      </c>
+      <c r="P21" s="55">
+        <f>SUM(H21,J21,L21,N21)/D21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="52" t="inlineStr">
+        <is>
+          <t>Self-managed by Majestic Realty — no 3rd-party management-fee GL line. Building 100% vacant all year; costs are pure carrying costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Majestic Commercenter Bldg 15</t>
+        </is>
+      </c>
+      <c r="B22" s="50" t="inlineStr">
+        <is>
+          <t>IND-WHSE</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="n">
+        <v>702491</v>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>100% (single tenant)</t>
+        </is>
+      </c>
+      <c r="H22" s="40" t="n">
+        <v>96706</v>
+      </c>
+      <c r="I22" s="54">
+        <f>H22/D22</f>
+        <v/>
+      </c>
+      <c r="J22" s="40" t="n">
+        <v>3616.47</v>
+      </c>
+      <c r="K22" s="54">
+        <f>J22/D22</f>
+        <v/>
+      </c>
+      <c r="L22" s="40" t="n">
+        <v>79483.92</v>
+      </c>
+      <c r="M22" s="54">
+        <f>L22/D22</f>
+        <v/>
+      </c>
+      <c r="N22" s="40" t="n">
+        <v>123015.72</v>
+      </c>
+      <c r="O22" s="54">
+        <f>N22/D22</f>
+        <v/>
+      </c>
+      <c r="P22" s="55">
+        <f>SUM(H22,J22,L22,N22)/D22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="52" t="inlineStr">
+        <is>
+          <t>Utilities landlord-side are minimal (Fire Service + a small 'Other' line) — consistent with a single-tenant NNN building where the tenant pays electricity/gas/water directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>NNN leases excluded from $/SF comps (tenant pays Insurance/Utilities/CAM/Management directly — no landlord-side actuals in the source documents)</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="n"/>
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="39" t="n"/>
+      <c r="E24" s="39" t="n"/>
+      <c r="F24" s="39" t="n"/>
+      <c r="G24" s="39" t="n"/>
+      <c r="H24" s="39" t="n"/>
+      <c r="I24" s="39" t="n"/>
+      <c r="J24" s="39" t="n"/>
+      <c r="K24" s="39" t="n"/>
+      <c r="L24" s="39" t="n"/>
+      <c r="M24" s="39" t="n"/>
+      <c r="N24" s="39" t="n"/>
+      <c r="O24" s="39" t="n"/>
+      <c r="P24" s="39" t="n"/>
+      <c r="Q24" s="39" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>DEN3 - Bull Crossing</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>R0198789</t>
+        </is>
+      </c>
+      <c r="Q25" s="52" t="inlineStr">
+        <is>
+          <t>NNN — Amazon pays all opex directly; landlord pro forma uses a blanket 5% expense load, not itemized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>DEN7</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>R0198530</t>
+        </is>
+      </c>
+      <c r="Q26" s="52" t="inlineStr">
+        <is>
+          <t>NNN — Amazon pays all opex directly; landlord pro forma uses a blanket 5% expense load, not itemized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
+        <is>
+          <t>DEN2 - PR Park 70</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="inlineStr">
+        <is>
+          <t>R0191292</t>
+        </is>
+      </c>
+      <c r="Q27" s="52" t="inlineStr">
+        <is>
+          <t>NNN — Amazon pays all opex directly; landlord pro forma uses a blanket 5% expense load, not itemized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>Home Depot Denver</t>
+        </is>
+      </c>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>R0180551</t>
+        </is>
+      </c>
+      <c r="Q28" s="52" t="inlineStr">
+        <is>
+          <t>NNN — Home Depot pays all opex directly; no landlord-side actual $ in the appeal package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="inlineStr">
+        <is>
+          <t>How to use: click any header and use Data &gt; Filter (or the AutoFilter arrows already enabled) to sort/filter by OCC Code or Size (SF) and build a comp set for a subject property of similar use and size. 'Basis' distinguishes actual-statement figures from the one proforma-assumption row (Shamrock Foods, owner-occupied). $/SF is blank ('n/a') where a $ amount exists but the property's building SF wasn't captured in Property Master, or where the category wasn't reported/applicable. OCC Code is a simple use-based classification inferred from each property's Property Type / Use in this database (IND-WHSE = industrial warehouse, IND-DIST = industrial distribution, IND-MFG = industrial manufacturing, IND-FLEX = industrial/flex, COM-MT = commercial multi-tenant) — it is NOT an official Adams County CAMA occupancy code; map/replace with the official code if one is needed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:Q22"/>
+  <mergeCells count="4">
+    <mergeCell ref="A24:Q24"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A30:Q30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add OCCC Code column and legend for filtering by property use type
- New "OCCC Legend" tab defines a short Occupancy Classification Code
  per distinct Property Type / Use.
- OCCC Code column added to Property Master, Income-Expense Summary,
  and Income-Expense Detail, derived from each property's existing
  Property Type / Use (no OCCC data existed in source docs or the
  prior workbook).
- AutoFilter enabled on all four tabs so line items, summary totals,
  and the property roster can be filtered to one use type.
- README documents the new tab, the code key, and notes this is an
  assigned classification pending confirmation of any official scheme.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEvYUU64sKrtpSq4tBAnfS
</commit_message>
<xml_diff>
--- a/Master_Property_Database.xlsx
+++ b/Master_Property_Database.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Documents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property Master" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenants &amp; Leases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments &amp; Valuation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income-Expense Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Parcels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Source Documents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="OCCC Legend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Property Master" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tenants &amp; Leases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assessments &amp; Valuation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Income-Expense Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Income-Expense Detail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Related Parcels" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OCCC Legend'!$A$4:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Property Master'!$A$4:$Z$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Income-Expense Summary'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Income-Expense Detail'!$A$4:$F$65</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -183,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -270,6 +276,8 @@
     <xf numFmtId="166" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -660,7 +668,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -970,7 +977,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -1010,7 +1016,164 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>OCCC CODE LEGEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>Occupancy Classification Codes -- assigned in this workbook from each property's Property Type / Use (Property Master tab). No such code existed in the source documents; rename/remap here if your organization uses a different OCCC scheme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OCCC Code</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Commercial (multi-tenant industrial)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Broadview</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Industrial - 2-unit (multi-tenant)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>5970 Marion Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>IND-DIST</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Industrial - Distribution</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>(7194) CO-Aurora</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>IND-FLEX</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Industrial / Flex (multi-tenant)</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Washington Business Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Industrial - Mfg / Food Processing</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>TempTee Brand Steaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>IND-WH</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Industrial - Warehouse</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>7205 Gilpin Way, SGS - Pennsylvania Industrial, 6770 E. 56th Ave</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:C10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1201,7 @@
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
     <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1054,7 +1218,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1179,6 +1342,11 @@
       <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>Source File</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>OCCC Code</t>
         </is>
       </c>
     </row>
@@ -1292,6 +1460,11 @@
           <t>R0178308.pdf</t>
         </is>
       </c>
+      <c r="Z5" s="6" t="inlineStr">
+        <is>
+          <t>IND-WH</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1401,6 +1574,11 @@
       <c r="Y6" s="6" t="inlineStr">
         <is>
           <t>R0169133.pdf</t>
+        </is>
+      </c>
+      <c r="Z6" s="6" t="inlineStr">
+        <is>
+          <t>IND-DIST</t>
         </is>
       </c>
     </row>
@@ -1508,6 +1686,11 @@
           <t>R0103792.pdf</t>
         </is>
       </c>
+      <c r="Z7" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1615,6 +1798,11 @@
           <t>5970 Marion P&amp;L/CF/xlsx</t>
         </is>
       </c>
+      <c r="Z8" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1726,6 +1914,11 @@
       <c r="Y9" s="6" t="inlineStr">
         <is>
           <t>5650_Washington_St.docx</t>
+        </is>
+      </c>
+      <c r="Z9" s="6" t="inlineStr">
+        <is>
+          <t>IND-FLEX</t>
         </is>
       </c>
     </row>
@@ -1835,6 +2028,11 @@
       <c r="Y10" s="6" t="inlineStr">
         <is>
           <t>R0024442.pdf</t>
+        </is>
+      </c>
+      <c r="Z10" s="6" t="inlineStr">
+        <is>
+          <t>IND-WH</t>
         </is>
       </c>
     </row>
@@ -1940,6 +2138,11 @@
           <t>R0002819.pdf</t>
         </is>
       </c>
+      <c r="Z11" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2051,17 +2254,23 @@
           <t>R0092302.pdf</t>
         </is>
       </c>
+      <c r="Z12" s="6" t="inlineStr">
+        <is>
+          <t>IND-WH</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:Z12"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A2:Z2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2100,7 +2309,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3143,7 +3351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3176,7 +3384,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -3385,7 +3592,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
@@ -3400,7 +3606,6 @@
       <c r="G12" s="20" t="n"/>
       <c r="H12" s="21" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
@@ -3597,7 +3802,6 @@
         <v>2460577</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -3625,13 +3829,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3639,6 +3843,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3655,7 +3860,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3680,6 +3884,11 @@
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Basis / Source</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>OCCC Code</t>
         </is>
       </c>
     </row>
@@ -3704,6 +3913,11 @@
           <t>5970_Marion 2024 P&amp;L (cash; incl. debt svc &amp; taxes)</t>
         </is>
       </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -3726,6 +3940,11 @@
           <t>2023 Cash Flow (cash; incl. debt svc &amp; taxes)</t>
         </is>
       </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -3747,6 +3966,11 @@
           <t>Owner-occupied; reported OpEx only ('in house' items = $0)</t>
         </is>
       </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -3769,6 +3993,11 @@
           <t>IRS Form 8825 (tax basis; incl. depreciation, amort. &amp; interest)</t>
         </is>
       </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="9"/>
     <row r="10" ht="28" customHeight="1">
@@ -3780,25 +4009,27 @@
       <c r="B10" s="20" t="n"/>
       <c r="C10" s="20" t="n"/>
       <c r="D10" s="20" t="n"/>
-      <c r="E10" s="21" t="n"/>
+      <c r="E10" s="20" t="n"/>
+      <c r="F10" s="21" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A4:F10"/>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3806,6 +4037,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3822,7 +4054,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3849,6 +4080,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>OCCC Code</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3874,6 +4110,11 @@
           <t>Whatever It Takes Transmissions + Integrated Turf Solutions</t>
         </is>
       </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3897,6 +4138,11 @@
       <c r="E6" s="6" t="inlineStr">
         <is>
           <t>CAM recoveries</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
         </is>
       </c>
     </row>
@@ -3925,6 +4171,11 @@
           <t>Printed total: $249,672.20.</t>
         </is>
       </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3946,6 +4197,11 @@
         <v>2175.55</v>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -3967,6 +4223,11 @@
         <v>394.3</v>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3988,6 +4249,11 @@
         <v>100</v>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -4009,6 +4275,11 @@
         <v>927.47</v>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -4030,6 +4301,11 @@
         <v>200</v>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -4055,6 +4331,11 @@
           <t>Deerwoods</t>
         </is>
       </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -4080,6 +4361,11 @@
           <t>net $0</t>
         </is>
       </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -4105,6 +4391,11 @@
           <t>Farmers</t>
         </is>
       </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -4130,6 +4421,11 @@
           <t>Adams Co.</t>
         </is>
       </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -4151,6 +4447,11 @@
         <v>800</v>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -4176,6 +4477,11 @@
           <t>Alpine Bank</t>
         </is>
       </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -4201,6 +4507,11 @@
           <t>Alpine Bank</t>
         </is>
       </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -4222,6 +4533,11 @@
         <v>465</v>
       </c>
       <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -4243,6 +4559,11 @@
         <v>293.68</v>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -4269,6 +4590,11 @@
           <t>Printed total: $162,774.36. cash basis; incl. debt service &amp; property taxes</t>
         </is>
       </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -4290,6 +4616,11 @@
         <v>89143.03999999999</v>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -4311,6 +4642,11 @@
         <v>523.01</v>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -4332,6 +4668,11 @@
         <v>500</v>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -4353,6 +4694,11 @@
         <v>157145.5</v>
       </c>
       <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -4379,6 +4725,11 @@
           <t>Printed total: $247,311.55.</t>
         </is>
       </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -4400,6 +4751,11 @@
         <v>1550</v>
       </c>
       <c r="E28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -4421,6 +4777,11 @@
         <v>47000</v>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -4442,6 +4803,11 @@
         <v>810</v>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -4463,6 +4829,11 @@
         <v>1016.31</v>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -4484,6 +4855,11 @@
         <v>2157.08</v>
       </c>
       <c r="E32" s="6" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -4505,6 +4881,11 @@
         <v>151.01</v>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -4526,6 +4907,11 @@
         <v>110</v>
       </c>
       <c r="E34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -4547,6 +4933,11 @@
         <v>6000</v>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -4568,6 +4959,11 @@
         <v>180</v>
       </c>
       <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -4589,6 +4985,11 @@
         <v>8640.99</v>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -4610,6 +5011,11 @@
         <v>37726.76</v>
       </c>
       <c r="E38" s="6" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -4631,6 +5037,11 @@
         <v>4968.83</v>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -4652,6 +5063,11 @@
         <v>26699.59</v>
       </c>
       <c r="E40" s="6" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -4673,6 +5089,11 @@
         <v>51624.89</v>
       </c>
       <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -4699,6 +5120,11 @@
           <t>Printed total: $188,635.46. cash basis; Owner Draw $100,000 (financing) excluded</t>
         </is>
       </c>
+      <c r="F42" s="18" t="inlineStr">
+        <is>
+          <t>IND-2U</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -4720,6 +5146,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -4741,6 +5172,11 @@
         <v>14050</v>
       </c>
       <c r="E44" s="6" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -4762,6 +5198,11 @@
         <v>10000</v>
       </c>
       <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -4787,6 +5228,11 @@
           <t>'in house'</t>
         </is>
       </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -4812,6 +5258,11 @@
           <t>'in house'</t>
         </is>
       </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -4833,6 +5284,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -4854,6 +5310,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="6" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -4875,6 +5336,11 @@
         <v>12000</v>
       </c>
       <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -4896,6 +5362,11 @@
         <v>102000</v>
       </c>
       <c r="E51" s="6" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -4922,6 +5393,11 @@
           <t>Printed total: $138,050.00. Adams Co. survey; 100% owner-occupied (~17,000 SF); 'in house' items = $0</t>
         </is>
       </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>IND-MFG</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -4945,6 +5421,11 @@
       <c r="E53" s="6" t="inlineStr">
         <is>
           <t>IRS Form 8825, Property A (125 Bridge St, COMMERCIAL)</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
         </is>
       </c>
     </row>
@@ -4973,6 +5454,11 @@
           <t>Printed total: $307,817.00.</t>
         </is>
       </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -4994,6 +5480,11 @@
         <v>776</v>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -5015,6 +5506,11 @@
         <v>12004</v>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -5036,6 +5532,11 @@
         <v>10211</v>
       </c>
       <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -5057,6 +5558,11 @@
         <v>98058</v>
       </c>
       <c r="E58" s="6" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -5078,6 +5584,11 @@
         <v>100279</v>
       </c>
       <c r="E59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -5099,6 +5610,11 @@
         <v>4731</v>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -5120,6 +5636,11 @@
         <v>47109</v>
       </c>
       <c r="E61" s="6" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -5141,6 +5662,11 @@
         <v>1080</v>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -5162,6 +5688,11 @@
         <v>2166</v>
       </c>
       <c r="E63" s="6" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -5183,6 +5714,11 @@
         <v>39767</v>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -5209,17 +5745,23 @@
           <t>Printed total: $316,181.00. IRS Form 8825; net rental loss $(8,364). Tax basis (incl. depreciation, amortization &amp; interest).</t>
         </is>
       </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>COM-MT</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:F65"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5249,7 +5791,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -5385,7 +5926,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>

</xml_diff>